<commit_message>
fix: ensure compare_jobs receives jobs argument and avoid redundant function call
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,7 +457,1326 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Visual Merchandiser</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/visual-merchandiser-at-zara-4364491240?position=1&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=I6CuO%2BXHoRyZAXx0jFIiNw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Department Manager</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/department-manager-at-zara-4364194840?position=2&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=NzFDuHtZAzMpYwR%2BMhUq9A%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Visual Merchandiser</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tampere</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/visual-merchandiser-at-zara-4363998069?position=3&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=ZiQE%2FaPjvCrymtFnELbAFQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Department Manager</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Tampere</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/department-manager-at-zara-4364481478?position=4&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=kIzzL%2Fo6qYDsf%2BsHJ%2FY5aA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Graphic Designer</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graphic-designer-at-ridge-4385561020?position=5&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=LuRn3k7DerJNY4SfZD%2FtQQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sales Assistant</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/sales-assistant-at-zara-4389603364?position=6&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=Nz1mJxcx2mlkjPTCwW5%2BYA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Researcher - Consumer Insights Games</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/researcher-consumer-insights-games-at-netflix-4362410898?position=7&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=H1ZDxRgD4IJPu4yaDKSJ%2Bw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sales Assistant</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tampere</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/sales-assistant-at-zara-4389192774?position=8&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=K9z%2FBZOZKySsnRJiaxIibA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Mindrift</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Freelance English Writer - AI Trainer</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/freelance-english-writer-ai-trainer-at-mindrift-4388295274?position=9&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=RaxdTnJR7OGKXu9SJKas%2FA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>YO IT Consulting</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Graphic Design - Remote</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graphic-design-remote-at-yo-it-consulting-4388617637?position=10&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=o7x%2FAxPW55r4yXISkklgag%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Medix Biochemica</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sales Director, North America &amp; Europe</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/sales-director-north-america-europe-at-medix-biochemica-4368713678?position=11&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=sWy4fNFxnuratEHt%2FXny5w%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>McKinsey &amp; Company</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/consultant-at-mckinsey-company-2679907113?position=12&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=kJE222uRWKb441Rfs6wFww%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Health &amp; Safety Advisor - Europe</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/health-safety-advisor-europe-at-crown-4370394451?position=13&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=ho6xZco2X33lhKCpSj7O9w%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/controller-at-jobgether-4388941890?position=14&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=eCwmyFtZjqzlMbZ2GXLnCg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Validia</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Lähihoitaja</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/l%C3%A4hihoitaja-at-validia-4388963187?position=15&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=RwQ8UTjE15HkstENRB7X0Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>betterhomes</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Real Estate Agent (Based in Dubai)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4376568688?position=16&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=M1VFxFOXiTJfC3x%2FUdTVxg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>betterhomes</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Real Estate Agent ( Based in Dubai)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Oulu</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373546207?position=17&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=gDruPJYsdB85P0Bo1GkTHw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>betterhomes</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Real Estate Agent ( Based in Dubai)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373524939?position=18&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=iNjhmC4GS8sXlxIWOVtqYQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Quality Manager</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/quality-manager-at-crown-4376585405?position=19&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=B7iIzSgUlR6Ko7SppRW1iA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sabik</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Managing Director (Europe and Africa)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Porvoo</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/managing-director-europe-and-africa-at-sabik-4390385199?position=20&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=mugmu5IukXrYuaKB8w8G8g%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Royal Caribbean Group</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Guest Service Officer</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/guest-service-officer-at-royal-caribbean-group-4379493842?position=21&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=n03OmlzOpbt8iMaDEZno%2Fw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>betterhomes</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Real Estate Agent ( Based in Dubai)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Tampere</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373543321?position=22&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=yeU8OVjLNFPN%2FpqicgFklQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>betterhomes</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Real Estate Agent ( Based in Dubai)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Turku</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373527919?position=23&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=XY44Rlexe%2FKuUWyvIFaENQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Quantity Surveyor - Europe</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/quantity-surveyor-europe-at-crown-4370502226?position=24&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=WsRVeTY7yxitvGe%2F%2B7an2Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Facilities Coordinator</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/facilities-coordinator-at-iceye-4366131126?position=25&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=5q974niKbhbwaBgRzdlgTA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Mindrift</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Machine Learning Developer (Freelance)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/machine-learning-developer-freelance-at-mindrift-4389448751?position=26&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=mkcgJCbTNUPPtMacj6kWvw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Logistics Specialist</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/logistics-specialist-at-iceye-4374724732?position=27&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=Mxn5yoJPCwY4kxzDtyKlXg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MultipleChat</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Professional Content Creator</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/professional-content-creator-at-multiplechat-4384141491?position=28&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=tPT1j9xXyVOYla1HvniTng%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Toloka Annotators</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Freelance Annotator (English) - AI Trainer</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/freelance-annotator-english-ai-trainer-at-toloka-annotators-4390619897?position=29&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=pMpBpi2gEGVCkGL2mFQZ6w%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Skeleton Technologies</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Production Planner (m/f/x)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Varkaus</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/production-planner-m-f-x-at-skeleton-technologies-4335958371?position=30&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=pxGGr3zWOlH98hd2jASh5A%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Emirates</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Helsinki Cabin Crew Opportunities (Dubai Based, Relocation Provided)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Helsinki Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/helsinki-cabin-crew-opportunities-dubai-based-relocation-provided-at-emirates-4386647938?position=31&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=twXXR2l4NTg3Zan%2FaCCLnQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Fazer</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Specialist, Digital Marketing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Vantaa</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/specialist-digital-marketing-at-fazer-4387933742?position=32&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=BHRyKDrBafdv9MGoaA9HQA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Skeleton Technologies</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Production Manager (m/f/x)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Varkaus</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/production-manager-m-f-x-at-skeleton-technologies-4335948513?position=33&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=q%2Fuo4khfgqN8%2B2iPTnljxQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DataTribe Collective</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Community Manager</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/social-media-community-manager-at-datatribe-collective-4390027743?position=34&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=sImqexCOCiowKpU9dXEv3Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Nbyula - Skillizens without Borders</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>International Student Ambassador - Study in Finland</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/international-student-ambassador-study-in-finland-at-nbyula-skillizens-without-borders-4257346845?position=35&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=llh1Nlu7m3T6yVfuiY9%2FgQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Arctic GM &amp; Sonka Resort | The Original Aurora Hunters®</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Other Jobs (Arctic GM &amp; Sonka Resort)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Rovaniemi</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/other-jobs-arctic-gm-sonka-resort-at-arctic-gm-sonka-resort-the-original-aurora-hunters%C2%AE-4383154558?position=36&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=bDDvPDng5DLD5w9ir0GGhg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>TSMG Holding</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Autonomous Vehicle Driver (T1 Certified)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/autonomous-vehicle-driver-t1-certified-at-tsmg-holding-4238599314?position=37&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=QQsty0NQOnASpYMq2AnzCg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Mindrift</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Freelance Management Consulting Partner (McKinsey / BCG / Bain)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/freelance-management-consulting-partner-mckinsey-bcg-bain-at-mindrift-4389047585?position=38&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=FQ5cEDiQGQHy2hW9BRsoxg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Hildén &amp; Kaira</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Freelancer-editoija (TikTok, Instagram, Youtube)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/freelancer-editoija-tiktok-instagram-youtube-at-hild%C3%A9n-kaira-4373547482?position=39&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=VDfH9TE%2B2Ki0O9MRRF90Bw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Comms8</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Media Assistant - Intern</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/media-assistant-intern-at-comms8-4365782976?position=40&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=c7yG7QNROqR%2F7soChU9UPA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Skeleton Technologies</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Senior Electrical Engineer (m/f/x)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Lappeenranta</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/senior-electrical-engineer-m-f-x-at-skeleton-technologies-4334399823?position=41&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=AmaGzWPjVY4U0dkKrqA%2F7w%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Homa</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Producer</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/producer-at-homa-4342662994?position=42&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=2RlMcoffAWdPMrJZdM0a9A%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Site Manager</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/site-manager-at-crown-4373937838?position=43&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=jQHSPrgkk21QrMAYusR28Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Customer Success Specialist with Coffee Experience</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/customer-success-specialist-with-coffee-experience-at-jobgether-4388938963?position=44&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=Hs5hp5C6Cr8i6X%2BiDJCLLw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>SOL ☀</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Kerääjä</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Vantaa</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/ker%C3%A4%C3%A4j%C3%A4-at-sol-%E2%98%80-4388786645?position=45&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=4JB1GHrZTFMgIYhSQcm0LQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Executive Producer, Live Services - Games</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/executive-producer-live-services-games-at-netflix-4374894857?position=46&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=t5XvzHopdh7ciMbWIVEkNQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Head of Logistics &amp; Freight Forwarding</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/head-of-logistics-freight-forwarding-at-iceye-4386734886?position=47&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=%2FFt2ZG71mnIAZh7jYAqiwQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Head of Customer Success</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/head-of-customer-success-at-jobgether-4388947651?position=48&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=9pVcpk99JBlhf8gz8FN%2BKg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Satellite Production Technician, Avionics</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/satellite-production-technician-avionics-at-iceye-4373827133?position=49&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=BU7wH6E0lXd5tbZTQWzPMA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Medix Biochemica</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Marketing Director</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/marketing-director-at-medix-biochemica-4362069234?position=50&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=A0Y5VCqbwISZFbRDD2zWvA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Senior Quality Manager (Construction)</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/senior-quality-manager-construction-at-crown-4373944606?position=51&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=X7MCU9sFVCZF3hCHxrQ2gA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Validia</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Tukipalvelutyöntekijä</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/tukipalveluty%C3%B6ntekij%C3%A4-at-validia-4388956475?position=52&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=KNu8rwlG%2FEkT9wR3eStmLQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Finance Business Partner - Corporate &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/finance-business-partner-corporate-operations-at-iceye-4332588706?position=53&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=pcqe9g4BAzZ1gQDpjmnGOg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Human Resources Business Partner</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/human-resources-business-partner-at-iceye-4377121889?position=54&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=wIIowSfefVPiJ1chVEA8rw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Skeleton Technologies</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Field Test Engineer (m/f/x)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Lappeenranta</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/field-test-engineer-m-f-x-at-skeleton-technologies-4371283030?position=55&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=QWLKQIhm9O471ASEmP4Yzg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Logistics Specialist</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/logistics-specialist-at-iceye-4384138498?position=56&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=k0HRZSDANliIbXtxU60oiw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Communications Manager, Nordics</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/marketing-communications-manager-nordics-at-iceye-4367462251?position=57&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=A%2Fjxmje85RnLKK95B7q96Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>YO IT Consulting</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Industrial Design - Remote</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/industrial-design-remote-at-yo-it-consulting-4389878792?position=58&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=dovwibtNUb8Ce3dMCWLBEQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Senior Manager Supply Chain, Strategy</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/senior-manager-supply-chain-strategy-at-iceye-4384874584?position=59&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=Dj6i%2FB9xYD2mpx%2BaDe8teQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>YO IT Consulting</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Creative Director - Remote</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/creative-director-remote-at-yo-it-consulting-4390494377?position=60&amp;pageNum=0&amp;refId=dW5YcHdXZ9NtgjITHhdo5w%3D%3D&amp;trackingId=uJtS3sTuz5s0%2FT9mDVHIQA%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: replace undefined Outlook reference with Application to enable email sending
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1777,6 +1777,1326 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Visual Merchandiser</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/visual-merchandiser-at-zara-4364491240?position=1&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=mQ9nfWgOQoSjF4G8173OGg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Department Manager</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/department-manager-at-zara-4364194840?position=2&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=074EU020Z3IqJCEHC42M4A%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Visual Merchandiser</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Tampere</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/visual-merchandiser-at-zara-4363998069?position=3&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=cUVzFueICXKoKsTZilCekg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Department Manager</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Tampere</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/department-manager-at-zara-4364481478?position=4&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=mHkmuZXviS6EDJ03LgBBnQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Graphic Designer</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graphic-designer-at-ridge-4385561020?position=5&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=sl61l6yLrKNHWJhpbTVrag%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Sales Assistant</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/sales-assistant-at-zara-4389603364?position=6&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=iLDKtflj6n%2BLAhZO%2FZ%2F7sA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Researcher - Consumer Insights Games</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/researcher-consumer-insights-games-at-netflix-4362410898?position=7&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=9pEZqbp7Bznu%2FAM3u1Rhfg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ZARA</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Sales Assistant</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Tampere</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/sales-assistant-at-zara-4389192774?position=8&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=2ucW9O5nSvCdg%2BTRcNUuQg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Mindrift</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Freelance English Writer - AI Trainer</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/freelance-english-writer-ai-trainer-at-mindrift-4388295274?position=9&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=FaM9W13Jk71oucTpzW%2B5Lg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>YO IT Consulting</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Graphic Design - Remote</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graphic-design-remote-at-yo-it-consulting-4388617637?position=10&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=XZdcXWgDtJfE4Vgiyr1qLQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Medix Biochemica</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Sales Director, North America &amp; Europe</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/sales-director-north-america-europe-at-medix-biochemica-4368713678?position=11&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=3saIOuIrOQ6VPYk8RiHi1Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>McKinsey &amp; Company</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Consultant</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/consultant-at-mckinsey-company-2679907113?position=12&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=S9YlhKwUQ7wVd8zNfR%2B8WQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Health &amp; Safety Advisor - Europe</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/health-safety-advisor-europe-at-crown-4370394451?position=13&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=XT%2BSCAB4%2ByKM3OjmJ0tfjw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Controller</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/controller-at-jobgether-4388941890?position=14&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=w9IocQWPQx7asfhlWQTARQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Validia</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Lähihoitaja</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/l%C3%A4hihoitaja-at-validia-4388963187?position=15&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=2iNCjdUvme2jc6RBq%2FIm6g%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>betterhomes</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Real Estate Agent (Based in Dubai)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4376568688?position=16&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=oMc4cLlQnfPX0pE%2FMGpOag%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>betterhomes</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Real Estate Agent ( Based in Dubai)</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Oulu</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373546207?position=17&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=5i7xR%2ByKw%2BLBWBmnWBYyuQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>betterhomes</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Real Estate Agent ( Based in Dubai)</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373524939?position=18&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=ovWI9n%2BTzftRCgVgj4%2F8YQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Quality Manager</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/quality-manager-at-crown-4376585405?position=19&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=oDJdgpOq%2FROBVwTdp7v%2FbQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Sabik</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Managing Director (Europe and Africa)</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Porvoo</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/managing-director-europe-and-africa-at-sabik-4390385199?position=20&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=BUNqrZrSv1iRe6XFp4Pfgg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Royal Caribbean Group</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Guest Service Officer</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/guest-service-officer-at-royal-caribbean-group-4379493842?position=21&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=I0aWPT6195woHktTz40PCw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>betterhomes</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Real Estate Agent ( Based in Dubai)</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Tampere</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373543321?position=22&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=Il4qc2ScCFCptalNOum14w%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>betterhomes</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Real Estate Agent ( Based in Dubai)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Turku</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373527919?position=23&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=hA3iaOTzMr00RvTDp3Hd%2Bg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Quantity Surveyor - Europe</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/quantity-surveyor-europe-at-crown-4370502226?position=24&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=3FKhgZthw9obvf2JiKyN3Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Facilities Coordinator</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/facilities-coordinator-at-iceye-4366131126?position=25&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=2WliV3e%2FD1lEUdfUIlLDew%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Mindrift</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Machine Learning Developer (Freelance)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/machine-learning-developer-freelance-at-mindrift-4389448751?position=26&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=KTc08UASoxUlmLfX%2BMzJMA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Logistics Specialist</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/logistics-specialist-at-iceye-4374724732?position=27&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=x8M72NULY5wcTaDVXKldxA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>MultipleChat</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Professional Content Creator</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/professional-content-creator-at-multiplechat-4384141491?position=28&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=fBMRHD%2FyjmYdKqjY7lWHAA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Toloka Annotators</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Freelance Annotator (English) - AI Trainer</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/freelance-annotator-english-ai-trainer-at-toloka-annotators-4390619897?position=29&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=N2fb%2Bsb%2F7Lm47nFJsux6lA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Skeleton Technologies</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Production Planner (m/f/x)</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Varkaus</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/production-planner-m-f-x-at-skeleton-technologies-4335958371?position=30&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=X1OfT5GBOenURWcEP4%2BpxQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Emirates</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Helsinki Cabin Crew Opportunities (Dubai Based, Relocation Provided)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Helsinki Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/helsinki-cabin-crew-opportunities-dubai-based-relocation-provided-at-emirates-4386647938?position=31&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=gAChpDT6%2FZzYCGuP2x2BcA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Fazer</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Specialist, Digital Marketing</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Vantaa</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/specialist-digital-marketing-at-fazer-4387933742?position=32&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=wub5yv27T%2BfEKN%2BVyWFurA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Skeleton Technologies</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Production Manager (m/f/x)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Varkaus</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/production-manager-m-f-x-at-skeleton-technologies-4335948513?position=33&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=JLnLVEio34dHtjlmJrPlmg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Nbyula - Skillizens without Borders</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>International Student Ambassador - Study in Finland</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/international-student-ambassador-study-in-finland-at-nbyula-skillizens-without-borders-4257346845?position=34&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=MxSiXsLQG%2B0r24ZceWMy0g%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>DataTribe Collective</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Social Media &amp; Community Manager</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/social-media-community-manager-at-datatribe-collective-4390027743?position=35&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=vPiL6nJLGnq4pt4%2FmE%2BLhw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Arctic GM &amp; Sonka Resort | The Original Aurora Hunters®</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Other Jobs (Arctic GM &amp; Sonka Resort)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Rovaniemi</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/other-jobs-arctic-gm-sonka-resort-at-arctic-gm-sonka-resort-the-original-aurora-hunters%C2%AE-4383154558?position=36&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=uG5QBcgpieQlQh1ePoJcTA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>TSMG Holding</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Autonomous Vehicle Driver (T1 Certified)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/autonomous-vehicle-driver-t1-certified-at-tsmg-holding-4238599314?position=37&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=5LpTArVvK3Rf4cIq6dcgdw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Mindrift</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Freelance Management Consulting Partner (McKinsey / BCG / Bain)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/freelance-management-consulting-partner-mckinsey-bcg-bain-at-mindrift-4389047585?position=38&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=XM6gLS6QGE49Y0drcWy%2BuA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Hildén &amp; Kaira</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Freelancer-editoija (TikTok, Instagram, Youtube)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/freelancer-editoija-tiktok-instagram-youtube-at-hild%C3%A9n-kaira-4373547482?position=39&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=nw33%2Fnnq%2BCHzKRpZ%2F35zPw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Comms8</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Media Assistant - Intern</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/media-assistant-intern-at-comms8-4365782976?position=40&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=3uiafRgc%2BaaA5kgdQAFFUw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Skeleton Technologies</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Senior Electrical Engineer (m/f/x)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Lappeenranta</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/senior-electrical-engineer-m-f-x-at-skeleton-technologies-4334399823?position=41&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=4Xu2i%2FrsgsrIKazUEHqZBA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Homa</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Producer</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/producer-at-homa-4342662994?position=42&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=pOf08NWnolwNmWd44SbPTA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Site Manager</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/site-manager-at-crown-4373937838?position=43&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=wa4rqhzBQ2bnIIPlGShJgQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>SOL ☀</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Kerääjä</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Vantaa</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/ker%C3%A4%C3%A4j%C3%A4-at-sol-%E2%98%80-4388786645?position=44&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=Wpjh7ExswY5F1tXizevgiQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Customer Success Specialist with Coffee Experience</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/customer-success-specialist-with-coffee-experience-at-jobgether-4388938963?position=45&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=IYIhoO1KQl1cijFRiGE%2B%2BA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Executive Producer, Live Services - Games</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/executive-producer-live-services-games-at-netflix-4374894857?position=46&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=9oNPliND9FhV3uMkcAY2YA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Head of Logistics &amp; Freight Forwarding</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/head-of-logistics-freight-forwarding-at-iceye-4386734886?position=47&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=xenwJYrtAa8J%2FHIY5bqU3A%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Head of Customer Success</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/head-of-customer-success-at-jobgether-4388947651?position=48&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=avLEOdYuLYFTZC3qPuMhJg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Satellite Production Technician, Avionics</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/satellite-production-technician-avionics-at-iceye-4373827133?position=49&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=O7JXXuvs2EFNmRdBIT6ilA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Medix Biochemica</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Marketing Director</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/marketing-director-at-medix-biochemica-4362069234?position=50&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=WD%2B2NN7YtpX250METEiW4A%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Crown</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Senior Quality Manager (Construction)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/senior-quality-manager-construction-at-crown-4373944606?position=51&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=I4QntMaUJa0BNiQpzj%2FcEA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Validia</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Tukipalvelutyöntekijä</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/tukipalveluty%C3%B6ntekij%C3%A4-at-validia-4388956475?position=52&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=QADz1ujT%2Ba611p5eZnbOvg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Finance Business Partner - Corporate &amp; Operations</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/finance-business-partner-corporate-operations-at-iceye-4332588706?position=53&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=gRNzWOxSSkA9sghSx%2FO2VA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Human Resources Business Partner</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/human-resources-business-partner-at-iceye-4377121889?position=54&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=TZiH9AvxMQC6jBnPcb9Y9Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>6G Flagship</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Director of International Affairs, International Affairs Office</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Oulu</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/director-of-international-affairs-international-affairs-office-at-6g-flagship-4389931663?position=55&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=USMpxTOsiJJCejSGZLyEgQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Skeleton Technologies</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Field Test Engineer (m/f/x)</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Lappeenranta</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/field-test-engineer-m-f-x-at-skeleton-technologies-4371283030?position=56&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=DPyhL0tnMG9wMvbp5yR6%2BQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Logistics Specialist</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/logistics-specialist-at-iceye-4384138498?position=57&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=0exU%2BK1AmnzVrpqsKJ%2BOPw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Communications Manager, Nordics</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/marketing-communications-manager-nordics-at-iceye-4367462251?position=58&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=gxOjDU4JEcr%2FzKAgn3fslw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>YO IT Consulting</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Industrial Design - Remote</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/industrial-design-remote-at-yo-it-consulting-4389878792?position=59&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=SIIn9GiJbTfZyRxk9Ni%2BOg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Senior Manager Supply Chain, Strategy</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/senior-manager-supply-chain-strategy-at-iceye-4384874584?position=60&amp;pageNum=0&amp;refId=TmudStJWQ9isxG5N12qRqw%3D%3D&amp;trackingId=w6jCc5BsykYBdHWHw6r%2FFA%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Text added README file
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -457,7 +457,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -474,7 +473,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/visual-merchandiser-at-zara-4364491240?position=1&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=o2zchxFOsRZgdxQ0pZnPhg%3D%3D</t>
@@ -497,7 +495,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/department-manager-at-zara-4364194840?position=2&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=ijaaXMiUUS8wu%2BENgairRg%3D%3D</t>
@@ -520,7 +517,6 @@
           <t>Tampere</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/visual-merchandiser-at-zara-4363998069?position=3&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=%2FXTrj5mUJcNZ6qnhZV7fFQ%3D%3D</t>
@@ -543,7 +539,6 @@
           <t>Tampere</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/department-manager-at-zara-4364481478?position=4&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=%2BtCRLgAZwj86fSBdE8B62Q%3D%3D</t>
@@ -566,7 +561,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/graphic-designer-at-ridge-4385561020?position=5&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=UHjnIbwNp97GzFmnS5ecgg%3D%3D</t>
@@ -589,7 +583,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/sales-assistant-at-zara-4389603364?position=6&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=VMnZcV%2FwjfZof7XRF%2FXpPA%3D%3D</t>
@@ -612,7 +605,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/researcher-consumer-insights-games-at-netflix-4362410898?position=7&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=VH0s4IasWqnPAZN56dHruA%3D%3D</t>
@@ -635,7 +627,6 @@
           <t>Tampere</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/sales-assistant-at-zara-4389192774?position=8&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=dX%2BVgmelbFJxsGNf3%2FNPug%3D%3D</t>
@@ -658,7 +649,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/freelance-english-writer-ai-trainer-at-mindrift-4388295274?position=9&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=JZg3Sch79xYSOt34ZBDajw%3D%3D</t>
@@ -681,7 +671,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/graphic-design-remote-at-yo-it-consulting-4388617637?position=10&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=QFK7hM1Hr9yEB5tLqb5lmA%3D%3D</t>
@@ -704,7 +693,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/sales-director-north-america-europe-at-medix-biochemica-4368713678?position=11&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=Nqatt%2F6X8LPegvRvltGOlQ%3D%3D</t>
@@ -727,7 +715,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/consultant-at-mckinsey-company-2679907113?position=12&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=EXcra7rTHjaecCeuZbyAzg%3D%3D</t>
@@ -750,7 +737,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/health-safety-advisor-europe-at-crown-4370394451?position=13&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=yJ6bEaWrHVRKv4ISV6RNEw%3D%3D</t>
@@ -773,7 +759,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/controller-at-jobgether-4388941890?position=14&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=qXrAPABhzh3ZM%2F66fcjfKw%3D%3D</t>
@@ -796,7 +781,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/l%C3%A4hihoitaja-at-validia-4388963187?position=15&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=WiyXrCeAhLJlo6Vs9HsDhg%3D%3D</t>
@@ -819,7 +803,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4376568688?position=16&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=vcmfeVTcAjKlhKunZCrKyw%3D%3D</t>
@@ -842,7 +825,6 @@
           <t>Oulu</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373546207?position=17&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=og6gfvoczsYUK1DAJZPSyg%3D%3D</t>
@@ -865,7 +847,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373524939?position=18&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=fwpHYOEga3Xce6s43uETNw%3D%3D</t>
@@ -888,7 +869,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/quality-manager-at-crown-4376585405?position=19&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=QkDErUrdPc4%2FkEcBT%2FKj9w%3D%3D</t>
@@ -911,7 +891,6 @@
           <t>Porvoo</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/managing-director-europe-and-africa-at-sabik-4390385199?position=20&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=76tAAQipin7LuCUjMIRZ0A%3D%3D</t>
@@ -934,7 +913,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/guest-service-officer-at-royal-caribbean-group-4379493842?position=21&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=1FlxijSzvobV76hIroufQg%3D%3D</t>
@@ -957,7 +935,6 @@
           <t>Tampere</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373543321?position=22&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=Ub6liM7AGGrVbIrIOa1Clg%3D%3D</t>
@@ -980,7 +957,6 @@
           <t>Turku</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/real-estate-agent-based-in-dubai-at-betterhomes-4373527919?position=23&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=H2qDL%2FoLolhtDiVP%2FKGGrw%3D%3D</t>
@@ -1003,7 +979,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/quantity-surveyor-europe-at-crown-4370502226?position=24&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=45wXAuO%2BMiEAJn7DYlVFaA%3D%3D</t>
@@ -1026,7 +1001,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/facilities-coordinator-at-iceye-4366131126?position=25&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=7s2%2F4GF0S7R839l77sd3Bg%3D%3D</t>
@@ -1049,7 +1023,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/machine-learning-developer-freelance-at-mindrift-4389448751?position=26&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=CBwMlNx%2F%2FWAopVLrqHhwQQ%3D%3D</t>
@@ -1072,7 +1045,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/logistics-specialist-at-iceye-4374724732?position=27&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=Y%2BL%2FmJFqDDnckxFWERuU%2FA%3D%3D</t>
@@ -1095,7 +1067,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/professional-content-creator-at-multiplechat-4384141491?position=28&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=4YdOZvb5LIavYjTkYW%2FZAA%3D%3D</t>
@@ -1118,7 +1089,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/freelance-annotator-english-ai-trainer-at-toloka-annotators-4390619897?position=29&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=sV8COAqMmhjlrjxfuCezVg%3D%3D</t>
@@ -1141,7 +1111,6 @@
           <t>Varkaus</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/production-planner-m-f-x-at-skeleton-technologies-4335958371?position=30&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=4kVgT7fIOvEmHwNmCC%2FLIg%3D%3D</t>
@@ -1164,7 +1133,6 @@
           <t>Helsinki Metropolitan Area</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/helsinki-cabin-crew-opportunities-dubai-based-relocation-provided-at-emirates-4386647938?position=31&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=ORT%2F6M%2B1x2tKz3wPGCkBdg%3D%3D</t>
@@ -1187,7 +1155,6 @@
           <t>Vantaa</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/specialist-digital-marketing-at-fazer-4387933742?position=32&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=lS%2BN6NcvHuxwH7JYIvdRuA%3D%3D</t>
@@ -1210,7 +1177,6 @@
           <t>Varkaus</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/production-manager-m-f-x-at-skeleton-technologies-4335948513?position=33&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=4vdGy%2FbocaNa0tJbq7CsFg%3D%3D</t>
@@ -1233,7 +1199,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/international-student-ambassador-study-in-finland-at-nbyula-skillizens-without-borders-4257346845?position=34&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=D%2B%2B6yOcAY1T747dj9elwag%3D%3D</t>
@@ -1256,7 +1221,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/social-media-community-manager-at-datatribe-collective-4390027743?position=35&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=fyqHXO0DUIloNZ1WgWTc6Q%3D%3D</t>
@@ -1279,7 +1243,6 @@
           <t>Rovaniemi</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/other-jobs-arctic-gm-sonka-resort-at-arctic-gm-sonka-resort-the-original-aurora-hunters%C2%AE-4383154558?position=36&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=9aGLILNiRIYE4dNrepnwtA%3D%3D</t>
@@ -1302,7 +1265,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/autonomous-vehicle-driver-t1-certified-at-tsmg-holding-4238599314?position=37&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=4ITZWrbHrNqgdY%2BNkJwwkQ%3D%3D</t>
@@ -1325,7 +1287,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/freelance-management-consulting-partner-mckinsey-bcg-bain-at-mindrift-4389047585?position=38&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=o%2FpD1EAO5UbuvF8YEG2pDg%3D%3D</t>
@@ -1348,7 +1309,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/freelancer-editoija-tiktok-instagram-youtube-at-hild%C3%A9n-kaira-4373547482?position=39&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=6ze4C%2BiY%2BkHJFcm6Dpz8eQ%3D%3D</t>
@@ -1371,7 +1331,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/media-assistant-intern-at-comms8-4365782976?position=40&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=FZ1EAmpMyNqYIVUG%2BzuKUQ%3D%3D</t>
@@ -1394,7 +1353,6 @@
           <t>Lappeenranta</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/senior-electrical-engineer-m-f-x-at-skeleton-technologies-4334399823?position=41&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=dWI0YSh3irQ54A5H2uAEEA%3D%3D</t>
@@ -1417,7 +1375,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/producer-at-homa-4342662994?position=42&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=pNUsL7GYy1sjxGwIMkG%2Bnw%3D%3D</t>
@@ -1440,7 +1397,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/site-manager-at-crown-4373937838?position=43&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=GyoH9DY8jmYD87LvNVFjNg%3D%3D</t>
@@ -1463,7 +1419,6 @@
           <t>Vantaa</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/ker%C3%A4%C3%A4j%C3%A4-at-sol-%E2%98%80-4388786645?position=44&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=R5KjReaZmHyWkzQPEr8PcA%3D%3D</t>
@@ -1486,7 +1441,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/customer-success-specialist-with-coffee-experience-at-jobgether-4388938963?position=45&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=hHnyYJVbsETqQtkBT6hU1Q%3D%3D</t>
@@ -1509,7 +1463,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/executive-producer-live-services-games-at-netflix-4374894857?position=46&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=2xvBPHiHrQDDXFJ7y6yo1w%3D%3D</t>
@@ -1532,7 +1485,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/head-of-logistics-freight-forwarding-at-iceye-4386734886?position=47&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=PA9WbTVmzYP7vPuKRrkh3w%3D%3D</t>
@@ -1555,7 +1507,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/head-of-customer-success-at-jobgether-4388947651?position=48&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=xL%2FKNrbvoYkq7BkQvlUCXQ%3D%3D</t>
@@ -1578,7 +1529,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/satellite-production-technician-avionics-at-iceye-4373827133?position=49&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=gn1hMubhCdr1PcaxD9CeYQ%3D%3D</t>
@@ -1601,7 +1551,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/marketing-director-at-medix-biochemica-4362069234?position=50&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=U4tEUD%2BbF7LhVt28Xggrng%3D%3D</t>
@@ -1624,7 +1573,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/senior-quality-manager-construction-at-crown-4373944606?position=51&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=GhvefCD7WFqg89rrfH6SjA%3D%3D</t>
@@ -1647,7 +1595,6 @@
           <t>Oulu</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/director-of-international-affairs-international-affairs-office-at-6g-flagship-4389931663?position=52&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=Mb%2BKLwZlIdZ40ii5qwYDaQ%3D%3D</t>
@@ -1670,7 +1617,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/tukipalveluty%C3%B6ntekij%C3%A4-at-validia-4388956475?position=53&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=NtejGptI8kF4agPqCawbYQ%3D%3D</t>
@@ -1693,7 +1639,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/finance-business-partner-corporate-operations-at-iceye-4332588706?position=54&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=ndjCs98MF4jCu6AMF0fN1A%3D%3D</t>
@@ -1716,7 +1661,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/human-resources-business-partner-at-iceye-4377121889?position=55&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=dXw0hSAEYcRSHOyFQHNWlw%3D%3D</t>
@@ -1739,7 +1683,6 @@
           <t>Lappeenranta</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/field-test-engineer-m-f-x-at-skeleton-technologies-4371283030?position=56&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=aIbB0bFVqGQMLmsFqpPw%2Fg%3D%3D</t>
@@ -1762,7 +1705,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/logistics-specialist-at-iceye-4384138498?position=57&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=bWy%2FMiZSDJoQfwxSObbHJQ%3D%3D</t>
@@ -1785,7 +1727,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/marketing-communications-manager-nordics-at-iceye-4367462251?position=58&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=a2x8z4pckzc%2FbshaNQdy5A%3D%3D</t>
@@ -1808,7 +1749,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/industrial-design-remote-at-yo-it-consulting-4389878792?position=59&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=i0UzcZ4VA0KGYZl%2BsG5gbQ%3D%3D</t>
@@ -1831,7 +1771,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/senior-manager-supply-chain-strategy-at-iceye-4384874584?position=60&amp;pageNum=0&amp;refId=1g%2FFpR6nSnEWqsD016D8%2Fg%3D%3D&amp;trackingId=lES96D9sjYhc2u1wppMiRA%3D%3D</t>

</xml_diff>

<commit_message>
Fix: Navigation and search logic, update robot.yaml entry point
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1777,6 +1777,1260 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Ericsson</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Software Developer Intern</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Kirkkonummi</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/software-developer-intern-at-ericsson-4383927574?position=1&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=v8Om8QTA8KxgvHV7Wzn9FA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>CaPS</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Summer Trainee</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-at-caps-4385029234?position=2&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=dGoMilq8ptF2FHr6MepN%2Fw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Fazer</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Fazer Graduate Program 2026 (Business, Finance and IT)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Vantaa</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/fazer-graduate-program-2026-business-finance-and-it-at-fazer-4385873665?position=3&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=w%2BqySqCWSwfajAYzhX%2B34g%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Nets</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Graduate Program IT &amp; Technology - Finland</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graduate-program-it-technology-finland-at-nets-4363583842?position=4&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=8ADEDNXIXNAykK0JhVU6Sg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Outokumpu</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Summer Trainee - IT</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Helsinki Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-it-at-outokumpu-4378158385?position=5&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=WlZx9jcry5o08Jf0nis%2F4w%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>VTT</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Join our student talent pool!</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/join-our-student-talent-pool%21-at-vtt-4347002215?position=6&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=MkG7XwNmaKDWCzVr4CamSg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Neste</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Summer Trainee, Communications</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-communications-at-neste-4387972509?position=7&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=E2Eiyhtn7XIhw8dN7Le0JQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Nets</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Graduate Program Product - Finland</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graduate-program-product-finland-at-nets-4366157902?position=8&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=VK8mvVbcjqUPuasBrgTKmw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Metso</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Trainee, IP &amp; Tech Legal</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/trainee-ip-tech-legal-at-metso-4387331764?position=9&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=qrMz83bysOOFGLw5w8LWfA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ASSA ABLOY Group</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Trainee - R&amp;D Engineer, Mechanics</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Joensuu</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/trainee-r-d-engineer-mechanics-at-assa-abloy-group-4353823734?position=10&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=jjGvhGBinWA7MqSXSIC4hQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>ASSA ABLOY Group</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Trainee - R&amp;D Engineer, Mechanics</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Joensuu</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/trainee-r-d-engineer-mechanics-at-assa-abloy-group-4353783875?position=11&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=S4t%2F7PxfA%2B5qnK3I55wT%2BQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Outokumpu</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Legal Trainee</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Helsinki Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/legal-trainee-at-outokumpu-4380268709?position=12&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=qU3hvmcsWpmgeXZLUpHgvw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Sense Valmennus Oy</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Myynti- ja markkinointiharjoittelija</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Helsinki Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/myynti-ja-markkinointiharjoittelija-at-sense-valmennus-oy-4386179215?position=13&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=Slm%2Bed0zU7xv4%2BMVR%2BWTWg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Dottir</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Junior Legal Trainee</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/junior-legal-trainee-at-dottir-4390573070?position=14&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=OaM8%2BaKi0oCdohR61UwKLQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>UPM</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Summer Trainee, Software Engineer Trainee, Decision Support and Advanced Analytics</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-software-engineer-trainee-decision-support-and-advanced-analytics-at-upm-4384152024?position=15&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=tNU3fqsc4QISYnLaJDWgEg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>GE Vernova</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>MSc Thesis Opportunities Through a Summer Internship – Multiple Openings</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Tampere</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/msc-thesis-opportunities-through-a-summer-internship-%E2%80%93-multiple-openings-at-ge-vernova-4389748568?position=16&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=9fsDslscf4W0flNQB%2ByUPw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Detection Technology</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Trainee, Application Engineer</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Oulu</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/trainee-application-engineer-at-detection-technology-4389843177?position=17&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=KmsmJEgvjClQci9OTf6MlQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Intern, Product Operations</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/intern-product-operations-at-iceye-4389745183?position=18&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=RiSSxQ0V5OYG5dlplzw3EA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Canonical</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Software Engineer - Python - Cloud - graduate level</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/software-engineer-python-cloud-graduate-level-at-canonical-4389955529?position=19&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=TxF4gr3HjKBqxNAqs08p%2FQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Kempower</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Summer Trainee - Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Greater Lahti Area</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-mechanical-engineering-at-kempower-4386317636?position=20&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=umsQiXzB%2FyA2bAfp4jjFwA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>European Investment Bank (EIB)</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Graduate Corporate - based in Luxembourg</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graduate-corporate-based-in-luxembourg-at-european-investment-bank-eib-4383821574?position=21&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=DUk6D%2BK2JO0KRinRbF8eRQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>SSH Communications Security</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Build Engineer Summer Trainee</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/build-engineer-summer-trainee-at-ssh-communications-security-4382893795?position=22&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=kleSGvf%2BV0VtrWsd5kj3bw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Mindrift</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Freelance Junior Journalist - AI Trainer</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/freelance-junior-journalist-ai-trainer-at-mindrift-4390329124?position=23&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=Vz1pJeVloaS8aXOZsUHiBA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Kempower</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Summer Trainee - Electrical Engineering</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Greater Lahti Area</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-electrical-engineering-at-kempower-4386326353?position=24&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=Wo8qu2rmi8vjsl%2FUIlEydA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>SSH Communications Security</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Test Automation Summer Trainee</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/test-automation-summer-trainee-at-ssh-communications-security-4382895784?position=25&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=bP7tC%2BGFDzM43eYeSeAJlA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Groundhawk.io</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Quality Assurance Summer Trainee</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/quality-assurance-summer-trainee-at-groundhawk-io-4387599827?position=26&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=t5N1wlEXuhq9fXMD0vUYtg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Nets</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Graduate Program Data Science &amp; Analytics - Finland</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graduate-program-data-science-analytics-finland-at-nets-4363583843?position=27&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=ysccZXwqDg7%2BW%2FYZbzLGOg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>6G Flagship</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>University trainee, 3 positons</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Oulu</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/university-trainee-3-positons-at-6g-flagship-4387808789?position=28&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=GVidXWy%2FVXfrkw01G3vtRQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Wolt</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Software Engineer</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/software-engineer-at-wolt-4380445640?position=29&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=KrOYEDw%2Fau4hmooHcb5Q%2FQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Nokia</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Machine Learning Research Intern, Bell Labs</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/machine-learning-research-intern-bell-labs-at-nokia-4383113951?position=30&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=qy6P0jQBxhvVi8%2F1NWbGGw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Winthrop Technologies</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Electrical Engineer Graduate - 2026</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/electrical-engineer-graduate-2026-at-winthrop-technologies-4354933815?position=32&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=eUx9zycv6vrDjz1PSb4Fcw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>GE HealthCare</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Summer intern – Test automation</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Kuopio</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-intern-%E2%80%93-test-automation-at-ge-healthcare-4375427664?position=33&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=fFn%2Bxo7IjYnG%2F%2FuRN7cF2Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Nets</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Graduate Program: Data Analyst Trainee</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Jyväskylä</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graduate-program-data-analyst-trainee-at-nets-4386358703?position=34&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=3uTBJtbkR%2BeLlw%2Fqe3cYLg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Orion Pharma</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Serialization Trainee</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/serialization-trainee-at-orion-pharma-4387095699?position=35&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=LtwHltAoid0KZ%2BCQ98AVZg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Orion Pharma</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Serialization Trainee</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Turku</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/serialization-trainee-at-orion-pharma-4387505149?position=36&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=FdEoTA3NWc70fGYKUqh0zw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Citycon</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Junior Financial Controller</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/junior-financial-controller-at-citycon-4387252865?position=37&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=MQqX0X7Rdv60ZV4X9ScpSw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Internship- Sales or Solution Engineering Paths-Espoo</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/internship-sales-or-solution-engineering-paths-espoo-at-salesforce-4389787242?position=38&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=Q67vMgaO4vtzm%2FPdNTkC%2Bg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Canonical</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Software Engineer - Python - Ubuntu Pro client - graduate level</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/software-engineer-python-ubuntu-pro-client-graduate-level-at-canonical-4233270755?position=39&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=vlZCKrzBA3LV04DumVPGug%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Supply Chain Specialist (Satellite Flight Control &amp; Structures category)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/supply-chain-specialist-satellite-flight-control-structures-category-at-iceye-4389471712?position=40&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=1Uc0WmyesuJUlh%2FfzYp29Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Ålandsbanken Abp</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Analyst Trainee</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Helsinki Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/analyst-trainee-at-%C3%A5landsbanken-abp-4382101215?position=41&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=AmBWaisXYUb5%2Bk8iWh8pvg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Nexi Group</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Graduate Program Finland - IT &amp; Technology (Junior QA Engineer)</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graduate-program-finland-it-technology-junior-qa-engineer-at-nexi-group-4356820317?position=42&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=dN7lT2bu1BvWxwSMS9Qr1Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Nets</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Graduate Program Marketing - Finland</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/graduate-program-marketing-finland-at-nets-4383307259?position=43&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=dMXty%2BP%2FDf3xi8SrVJre3g%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>ICEYE</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Lab Technician</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/lab-technician-at-iceye-4380931924?position=45&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=rkm0trlk1%2FkZdAc8WSg7Aw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Nokia</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Summer Trainee in Direct Production</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Oulu</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-in-direct-production-at-nokia-4352910259?position=46&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=%2FTSMAizJ5RmXOJBJNichQA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Kempower</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Summer Trainee - Commercial Excellence</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Helsinki Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-commercial-excellence-at-kempower-4382951511?position=47&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=X1DnSwoEcVfhK9iT3g98eQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Kempower</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Summer Trainee - Commercial Excellence</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Greater Lahti Area</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-commercial-excellence-at-kempower-4382951510?position=49&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=lx6EtM2LMuJgPokYaieMyg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Mercury</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Junior Civil Engineer</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/junior-civil-engineer-at-mercury-4344388754?position=50&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=52CJeTrCZ0m8GAY7%2FwdT6w%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Physics World</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Quantum computer calibration intern</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/quantum-computer-calibration-intern-at-physics-world-4387156475?position=51&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=eGhNZ%2FPjukhpKMbw4KJ6IA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Ivy</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Finance &amp; Operations Working Student (m/f/d)</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/finance-operations-working-student-m-f-d-at-ivy-4387839727?position=52&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=BgjBJ5nGwAKjp0qlEeo%2Fmw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Wolt</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Program Manager, Technology &amp; Insights (EMEA)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/program-manager-technology-insights-emea-at-wolt-4368244864?position=53&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=cvmehYzsyEsNPdGH3811Pg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Ahlstrom</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Summer Trainee Procurement Specialist</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Tampere</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-procurement-specialist-at-ahlstrom-4374032395?position=54&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=BaQxYdk2u3GmDSFMbiV2sA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Siemens</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Solution Engineer Trainee #FutureWerner</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/solution-engineer-trainee-%23futurewerner-at-siemens-4385381651?position=55&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=Tlxn%2B7%2FU5DirrVoXVlFMJQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Mindrift</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Junior Linguistics Expert - Freelance AI Trainer</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/junior-linguistics-expert-freelance-ai-trainer-at-mindrift-4390313876?position=56&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=cCA1OHUX0boHY4VEKVBKAA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>VEO Group</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Työharjoittelu VEOn tuotannossa / Praktik i VEO produktion / Internship at the VEO factory</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Vaasa</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/ty%C3%B6harjoittelu-veon-tuotannossa-praktik-i-veo-produktion-internship-at-the-veo-factory-at-veo-group-4106255126?position=57&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=fs7ESHBgw0%2FjuCKYT779SA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Wolt</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Program Manager - Recruiting Programs, Internships &amp; Emerging Talent</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/program-manager-recruiting-programs-internships-emerging-talent-at-wolt-4372329398?position=58&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=N5mpq5LUzgaIduZMstdwzQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Lantmännen Unibake</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Global Graduate Program: Supply Chain &amp; Production</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/global-graduate-program-supply-chain-production-at-lantm%C3%A4nnen-unibake-4366781135?position=59&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=km0qFl6GhoXOiS%2BM2xInew%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Cadmatic</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Junior Cloud Specialist</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/junior-cloud-specialist-at-cadmatic-4386755804?position=60&amp;pageNum=0&amp;refId=3pRG3SSG5SI2gwxy5t4Y7w%3D%3D&amp;trackingId=WttL1Aa%2F9lFjpuoS65bHsw%3D%3D</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix extraction loop (count), remove duplicate keywords, and move teardown to end
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,7 +457,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -474,7 +473,6 @@
           <t>Helsinki Metropolitan Area</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-it-at-outokumpu-4378158385?position=1&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=AgJDpPV1vI3tzemc9IFf4Q%3D%3D</t>
@@ -497,7 +495,6 @@
           <t>Kirkkonummi</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/software-developer-intern-at-ericsson-4383927574?position=2&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=RZVwzJSKTdUs7AapLfiShw%3D%3D</t>
@@ -520,7 +517,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/fy26-engineering-intern-%E2%80%93-systems-software-engineering-espoo-finland-at-qualcomm-4391200030?position=3&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=Mi%2FFK8bXtSnvNWxiffmk4A%3D%3D</t>
@@ -543,7 +539,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-software-engineer-trainee-decision-support-and-advanced-analytics-at-upm-4384152024?position=4&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=f4ahbO%2FnYbQACEBgSFyj8w%3D%3D</t>
@@ -566,7 +561,6 @@
           <t>Helsinki Metropolitan Area</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/legal-trainee-at-outokumpu-4380268709?position=5&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=LIB%2FPGl%2BQ%2BWqI8yO3CjEyA%3D%3D</t>
@@ -589,7 +583,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/data-automation-trainee-at-orion-pharma-4392771091?position=6&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=tnG43gotG9aBqphTuko3OQ%3D%3D</t>
@@ -612,7 +605,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/forward-deployed-ai-software-engineer-internship-finland-bcg-x-at-bcg-x-4389310249?position=7&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=Pmj3GmtrsGfMYxml%2BfoUUA%3D%3D</t>
@@ -635,7 +627,6 @@
           <t>Greater Lahti Area</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-electrical-engineering-at-kempower-4386326353?position=8&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=H8YEcNGwE0k3OW0uJPp3vQ%3D%3D</t>
@@ -658,7 +649,6 @@
           <t>Greater Lahti Area</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-mechanical-engineer-at-kempower-4391768387?position=9&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=OZ5lUkQ3Fl6rIMJPiOR%2F%2BA%3D%3D</t>
@@ -681,7 +671,6 @@
           <t>Greater Lahti Area</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-mechanical-engineering-at-kempower-4386317636?position=10&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=gLvs7zhYJFWilwKXBVY6%2Bg%3D%3D</t>
@@ -704,7 +693,6 @@
           <t>Oulu</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-in-direct-production-at-nokia-4352910259?position=11&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=fPXWX49OlIAT7ektfzuHvw%3D%3D</t>
@@ -727,7 +715,6 @@
           <t>Hämeenlinna</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-system-specialist-at-huhtamaki-4387993415?position=12&amp;pageNum=0&amp;refId=y5VM40q%2FXFFjXe3an7tulQ%3D%3D&amp;trackingId=LRU0oQG0iO375iFVL2MV8g%3D%3D</t>
@@ -750,7 +737,6 @@
           <t>Helsinki Metropolitan Area</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-it-at-outokumpu-4378158385?position=1&amp;pageNum=0&amp;refId=Nb1QPcBcDcsSrfMDcSZvhA%3D%3D&amp;trackingId=KfVeVRzeGP%2B7eykt8Sz%2FAA%3D%3D</t>
@@ -773,7 +759,6 @@
           <t>Kirkkonummi</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/software-developer-intern-at-ericsson-4383927574?position=2&amp;pageNum=0&amp;refId=Nb1QPcBcDcsSrfMDcSZvhA%3D%3D&amp;trackingId=GL0IPlzPOQcNkNF6B6ym8w%3D%3D</t>
@@ -796,7 +781,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/fy26-engineering-intern-%E2%80%93-systems-software-engineering-espoo-finland-at-qualcomm-4391200030?position=3&amp;pageNum=0&amp;refId=Nb1QPcBcDcsSrfMDcSZvhA%3D%3D&amp;trackingId=xu%2BPCpJpbBMTzC4N%2FQ5OHQ%3D%3D</t>
@@ -819,7 +803,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-software-engineer-trainee-decision-support-and-advanced-analytics-at-upm-4384152024?position=4&amp;pageNum=0&amp;refId=Nb1QPcBcDcsSrfMDcSZvhA%3D%3D&amp;trackingId=3g%2FQS3OxB2Y3n60dF4diEg%3D%3D</t>
@@ -842,7 +825,6 @@
           <t>Jakobstad</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/ty%C3%B6harjoittelu-l%C3%A4hituki-pietarsaari-at-tiera-oy-4386726918?position=5&amp;pageNum=0&amp;refId=Nb1QPcBcDcsSrfMDcSZvhA%3D%3D&amp;trackingId=7Fdiawu5T%2F5omEiDSUtncw%3D%3D</t>
@@ -865,7 +847,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/forward-deployed-ai-software-engineer-internship-finland-bcg-x-at-bcg-x-4389310249?position=6&amp;pageNum=0&amp;refId=Nb1QPcBcDcsSrfMDcSZvhA%3D%3D&amp;trackingId=7yRUFjGJk6Nic0qjPsF5yQ%3D%3D</t>
@@ -888,7 +869,6 @@
           <t>Helsinki Metropolitan Area</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-it-at-outokumpu-4378158385?position=1&amp;pageNum=0&amp;refId=kSgMG3kshZRPw8227jyzgw%3D%3D&amp;trackingId=AvocjhlE8ONhV36htbVnHg%3D%3D</t>
@@ -911,7 +891,6 @@
           <t>Kirkkonummi</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/software-developer-intern-at-ericsson-4383927574?position=2&amp;pageNum=0&amp;refId=kSgMG3kshZRPw8227jyzgw%3D%3D&amp;trackingId=3aF6iW4t2ScVaZOA845fnw%3D%3D</t>
@@ -934,7 +913,6 @@
           <t>Finland</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/fy26-engineering-intern-%E2%80%93-systems-software-engineering-espoo-finland-at-qualcomm-4391200030?position=3&amp;pageNum=0&amp;refId=kSgMG3kshZRPw8227jyzgw%3D%3D&amp;trackingId=%2BgakYcDTlrdZpm1bj4DXQA%3D%3D</t>
@@ -957,7 +935,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-software-engineer-trainee-decision-support-and-advanced-analytics-at-upm-4384152024?position=4&amp;pageNum=0&amp;refId=kSgMG3kshZRPw8227jyzgw%3D%3D&amp;trackingId=3eE%2FotI7LiHJmnv%2F%2BDg6AQ%3D%3D</t>
@@ -980,7 +957,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/forward-deployed-ai-software-engineer-internship-finland-bcg-x-at-bcg-x-4389310249?position=5&amp;pageNum=0&amp;refId=kSgMG3kshZRPw8227jyzgw%3D%3D&amp;trackingId=3%2FFZLXMwFhWtW0NyFtH2mA%3D%3D</t>
@@ -1003,7 +979,6 @@
           <t>Hämeenlinna</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-system-specialist-at-huhtamaki-4387993415?position=6&amp;pageNum=0&amp;refId=kSgMG3kshZRPw8227jyzgw%3D%3D&amp;trackingId=QULulSQgjQH9kXFyHZR9wQ%3D%3D</t>
@@ -1026,7 +1001,6 @@
           <t>Kirkkonummi</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/software-developer-intern-at-ericsson-4383927574?position=1&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=IBxb%2BvyarvNV29TS7Jixcw%3D%3D</t>
@@ -1049,7 +1023,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/intern-product-operations-at-iceye-4389745183?position=2&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=9mJV8OsCVil1DlO8I4VC7w%3D%3D</t>
@@ -1072,7 +1045,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/satellite-production-technician-avionics-at-iceye-4373827133?position=3&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=tv4B%2FlkeG191J%2FboJbx87Q%3D%3D</t>
@@ -1095,7 +1067,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/logistics-specialist-at-iceye-4374724732?position=4&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=ZxO8QTBF9wQWggatoQPJmA%3D%3D</t>
@@ -1118,7 +1089,6 @@
           <t>Kuopio</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-intern-%E2%80%93-test-automation-at-ge-healthcare-4375427664?position=5&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=8YM661BX9Lkkgjtvp%2BEWGQ%3D%3D</t>
@@ -1141,7 +1111,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/logistics-specialist-at-iceye-4384138498?position=6&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=ahwB7Y4EViiFJ3xWI92cCg%3D%3D</t>
@@ -1164,7 +1133,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/supply-chain-specialist-satellite-flight-control-structures-category-at-iceye-4389471712?position=7&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=kFihZtVAr0bnOSoR3zdYng%3D%3D</t>
@@ -1187,7 +1155,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/hr-intern-at-huawei-4391224246?position=8&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=Q7aoyCIXpNBlT5vQ0wtlNw%3D%3D</t>
@@ -1210,7 +1177,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/hr-summer-intern-at-virta-ltd-4390953239?position=9&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=UG4%2FuBVQ%2FNnAWhH50%2FCupQ%3D%3D</t>
@@ -1233,7 +1199,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-communications-at-neste-4387972509?position=10&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=xZ%2FAnQbccqWJ5rkniPFq%2BQ%3D%3D</t>
@@ -1256,7 +1221,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/internship-sales-or-solution-engineering-paths-espoo-at-salesforce-4389787242?position=11&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=DsdB3AMaPl91aBj8e5vYzA%3D%3D</t>
@@ -1279,7 +1243,6 @@
           <t>Oulu</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/university-trainee-3-positons-at-6g-flagship-4387808789?position=12&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=aQn9BJVrZN0PyAGz2d%2FRGg%3D%3D</t>
@@ -1302,7 +1265,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/lab-technician-at-iceye-4380931924?position=13&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=l2Vz3fhnGMsTKu8JIHUGiA%3D%3D</t>
@@ -1325,7 +1287,6 @@
           <t>Helsinki Metropolitan Area</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/office-operations-intern-at-supercell-4391540758?position=14&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=QvWnMRbW3ZfQueElKfFjyg%3D%3D</t>
@@ -1348,7 +1309,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/quantum-technology-and-software-development-internships-qpu-performance-group-at-iqm-quantum-computers-4343365600?position=15&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=6EUSewJ4rUP9in9tnHhyIA%3D%3D</t>
@@ -1371,7 +1331,6 @@
           <t>Vaasa</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/get-to-know-technology-2026-internship-program-in-vaasa-at-w%C3%A4rtsil%C3%A4-4384135595?position=16&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=1FT7L5F4ypkCiV6eApUzSw%3D%3D</t>
@@ -1394,7 +1353,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/junior-legal-trainee-at-dottir-4390573070?position=17&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=LM1YskmSgwYWdSB8Kw%2F0Ag%3D%3D</t>
@@ -1417,7 +1375,6 @@
           <t>Vantaa</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/operations-early-talent-leadership-development-program-2026-intake-pre-registration-at-eaton-4326640078?position=18&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=nx0cGeAv6J39POgtbv2KLw%3D%3D</t>
@@ -1440,7 +1397,6 @@
           <t>Oulu</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/university-teacher-epidemiology-and-biomedical-data-science-faculty-of-medicine-at-6g-flagship-4380025507?position=19&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=1U5RLOklEGCRJJdfuVBxzw%3D%3D</t>
@@ -1463,7 +1419,6 @@
           <t>Espoo</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/summer-trainee-2026-financial-energy-analyst-elron-at-elomatic-4385795514?position=20&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=Ib9HrB6lgYcSJKMo0DM3xQ%3D%3D</t>
@@ -1486,7 +1441,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/global-graduate-program-supply-chain-production-at-lantm%C3%A4nnen-unibake-4366781135?position=21&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=li7ZAnTPym3xdfpjKE6mtg%3D%3D</t>
@@ -1509,7 +1463,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/account-management-working-student-finland-at-nordex-group-4385523408?position=22&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=h%2FUPcjODuYagvPORF8P%2Bdw%3D%3D</t>
@@ -1532,7 +1485,6 @@
           <t>Vantaa</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/services-sales-operations-talent-leadership-development-program-at-eaton-4392659433?position=23&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=Km87wkTWngAZxuq7qkayGQ%3D%3D</t>
@@ -1555,7 +1507,6 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/forward-deployed-ai-scientist-internship-finland-bcg-x-at-bcg-x-4388999814?position=24&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=bHbQzM8U1mTyrTtrOyiWcA%3D%3D</t>
@@ -1578,10 +1529,78 @@
           <t>Helsinki</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>https://fi.linkedin.com/jobs/view/forward-deployed-ai-software-engineer-internship-finland-bcg-x-at-bcg-x-4389310249?position=25&amp;pageNum=0&amp;refId=8gkZXf89E9Ez8FI%2BI18Qkw%3D%3D&amp;trackingId=Kww4azhoAS8%2F7DptqIv8GA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Kemira</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Summer Trainee, Finance</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Helsinki Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/summer-trainee-finance-at-kemira-4395136677?position=5&amp;pageNum=0&amp;refId=dYxYQCZIkTG08k0I3iStlA%3D%3D&amp;trackingId=hC2PTpsKAhhVIBAdJsgWnw%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>KPMG Finland</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Strategy Consultant Trainee</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Helsinki Metropolitan Area</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/strategy-consultant-trainee-at-kpmg-finland-4395002636?position=14&amp;pageNum=0&amp;refId=dYxYQCZIkTG08k0I3iStlA%3D%3D&amp;trackingId=5cU%2BV%2FENJVamdxNMeFG0ZA%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Symphony of views</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Project Intern</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Helsinki</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://fi.linkedin.com/jobs/view/project-intern-at-symphony-of-views-4352696229?position=3&amp;pageNum=0&amp;refId=vyA3p4Qn48JWsFa%2Fqq531g%3D%3D&amp;trackingId=%2BNBJlWCE0GBDLTP%2Fk9%2FXNg%3D%3D</t>
         </is>
       </c>
     </row>

</xml_diff>